<commit_message>
Update sales brainstorm items: know-how differentiator, Cestto case
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ld9Fj63CqEHYrhnAJFn4Xb
</commit_message>
<xml_diff>
--- a/ledwave-comercial/LedWave_Playbook_Comercial_Nichos.xlsx
+++ b/ledwave-comercial/LedWave_Playbook_Comercial_Nichos.xlsx
@@ -852,13 +852,13 @@
     <t xml:space="preserve">Ano de fundação + vida útil dos painéis</t>
   </si>
   <si>
-    <t xml:space="preserve">No hall</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[Descrever com o comercial]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[Definir]</t>
+    <t xml:space="preserve">Know-how</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mais de 15 anos fabricando, instalando e operando painéis de LED: sabemos o que funciona em cada tipo de espaço, do PDV ao maior painel da América Latina.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Histórico de projetos + Boulevard.Live</t>
   </si>
   <si>
     <t xml:space="preserve">Prova social</t>
@@ -1032,10 +1032,10 @@
     <t xml:space="preserve">Beto Carrero World</t>
   </si>
   <si>
-    <t xml:space="preserve">Cesstto</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[Confirmar nome e segmento]</t>
+    <t xml:space="preserve">Cestto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[Confirmar segmento]</t>
   </si>
   <si>
     <t xml:space="preserve">Museu do Amanhã</t>
@@ -14422,7 +14422,7 @@
       </c>
       <c r="E10" s="22"/>
     </row>
-    <row r="11" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="12" t="s">
         <v>269</v>
       </c>
@@ -14433,7 +14433,7 @@
         <v>271</v>
       </c>
       <c r="D11" s="22" t="s">
-        <v>265</v>
+        <v>254</v>
       </c>
       <c r="E11" s="22"/>
     </row>

</xml_diff>

<commit_message>
Apply LedWave visual identity: official logo, brand palette, LED dot motif
Decks now use the official logo on light layouts, the logo's gray and the
cyan-to-magenta LED gradient; workbooks use the same palette. CLAUDE.md
records the rule to always use the official logo.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ld9Fj63CqEHYrhnAJFn4Xb
</commit_message>
<xml_diff>
--- a/ledwave-comercial/LedWave_Playbook_Comercial_Nichos.xlsx
+++ b/ledwave-comercial/LedWave_Playbook_Comercial_Nichos.xlsx
@@ -4142,7 +4142,7 @@
     <font>
       <b val="true"/>
       <sz val="11"/>
-      <color rgb="FF1B1340"/>
+      <color rgb="FF3D3D3D"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -4171,7 +4171,7 @@
     <font>
       <i val="true"/>
       <sz val="10"/>
-      <color rgb="FFC2185B"/>
+      <color rgb="FF8A5CF6"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -4193,7 +4193,7 @@
     <font>
       <b val="true"/>
       <sz val="10"/>
-      <color rgb="FFC2185B"/>
+      <color rgb="FF8A5CF6"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -4201,7 +4201,7 @@
     <font>
       <i val="true"/>
       <sz val="9"/>
-      <color rgb="FFC2185B"/>
+      <color rgb="FF8A5CF6"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -4209,7 +4209,7 @@
     <font>
       <b val="true"/>
       <sz val="12"/>
-      <color rgb="FF1B1340"/>
+      <color rgb="FF3D3D3D"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -4224,8 +4224,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF1B1340"/>
-        <bgColor rgb="FF000000"/>
+        <fgColor rgb="FF3D3D3D"/>
+        <bgColor rgb="FF333300"/>
       </patternFill>
     </fill>
     <fill>
@@ -4236,19 +4236,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFC2185B"/>
-        <bgColor rgb="FFB00020"/>
+        <fgColor rgb="FF8A5CF6"/>
+        <bgColor rgb="FF9999FF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF5F5F7"/>
-        <bgColor rgb="FFFFFFFF"/>
+        <bgColor rgb="FFF2F3F7"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFEDE7F6"/>
+        <fgColor rgb="FFF2F3F7"/>
         <bgColor rgb="FFF5F5F7"/>
       </patternFill>
     </fill>
@@ -4496,7 +4496,7 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFC2185B"/>
+          <fgColor rgb="FF8A5CF6"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -4565,9 +4565,9 @@
       <rgbColor rgb="FFD0CCE0"/>
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
-      <rgbColor rgb="FFC2185B"/>
+      <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FFFFF8D6"/>
-      <rgbColor rgb="FFF5F5F7"/>
+      <rgbColor rgb="FFF2F3F7"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
       <rgbColor rgb="FF0066CC"/>
@@ -4581,7 +4581,7 @@
       <rgbColor rgb="FF008080"/>
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FF00CCFF"/>
-      <rgbColor rgb="FFEDE7F6"/>
+      <rgbColor rgb="FFF5F5F7"/>
       <rgbColor rgb="FFD7F2DF"/>
       <rgbColor rgb="FFFFFF99"/>
       <rgbColor rgb="FF99CCFF"/>
@@ -4594,7 +4594,7 @@
       <rgbColor rgb="FFFFCC00"/>
       <rgbColor rgb="FFFF9900"/>
       <rgbColor rgb="FFFF6600"/>
-      <rgbColor rgb="FF666699"/>
+      <rgbColor rgb="FF8A5CF6"/>
       <rgbColor rgb="FF999999"/>
       <rgbColor rgb="FF003366"/>
       <rgbColor rgb="FF339966"/>
@@ -4603,7 +4603,7 @@
       <rgbColor rgb="FF993300"/>
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FF333399"/>
-      <rgbColor rgb="FF1B1340"/>
+      <rgbColor rgb="FF3D3D3D"/>
     </indexedColors>
   </colors>
 </styleSheet>
@@ -4803,7 +4803,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <tabColor rgb="FFC2185B"/>
+    <tabColor rgb="FF8A5CF6"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D16"/>
@@ -4937,7 +4937,7 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <tabColor rgb="FF1B1340"/>
+    <tabColor rgb="FF3D3D3D"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E39"/>
@@ -5408,7 +5408,7 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <tabColor rgb="FF1B1340"/>
+    <tabColor rgb="FF3D3D3D"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F62"/>
@@ -6260,7 +6260,7 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <tabColor rgb="FF1B1340"/>
+    <tabColor rgb="FF3D3D3D"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D68"/>
@@ -6969,7 +6969,7 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <tabColor rgb="FF1B1340"/>
+    <tabColor rgb="FF3D3D3D"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E33"/>
@@ -7419,7 +7419,7 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <tabColor rgb="FF1B1340"/>
+    <tabColor rgb="FF3D3D3D"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:C21"/>
@@ -7636,7 +7636,7 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <tabColor rgb="FFC2185B"/>
+    <tabColor rgb="FF8A5CF6"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E54"/>
@@ -8294,7 +8294,7 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <tabColor rgb="FF1B1340"/>
+    <tabColor rgb="FF3D3D3D"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D19"/>
@@ -8573,7 +8573,7 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <tabColor rgb="FFC2185B"/>
+    <tabColor rgb="FF8A5CF6"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:M305"/>
@@ -12975,7 +12975,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <tabColor rgb="FFC2185B"/>
+    <tabColor rgb="FF8A5CF6"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F19"/>
@@ -13331,7 +13331,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <tabColor rgb="FF1B1340"/>
+    <tabColor rgb="FF3D3D3D"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G12"/>
@@ -13601,7 +13601,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <tabColor rgb="FF1B1340"/>
+    <tabColor rgb="FF3D3D3D"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F18"/>
@@ -13939,7 +13939,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <tabColor rgb="FFC2185B"/>
+    <tabColor rgb="FF8A5CF6"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F22"/>
@@ -14269,7 +14269,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <tabColor rgb="FFC2185B"/>
+    <tabColor rgb="FF8A5CF6"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E22"/>
@@ -14624,7 +14624,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <tabColor rgb="FFC2185B"/>
+    <tabColor rgb="FF8A5CF6"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:I19"/>
@@ -14936,7 +14936,7 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <tabColor rgb="FFC2185B"/>
+    <tabColor rgb="FF8A5CF6"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:Y21"/>
@@ -16407,7 +16407,7 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <tabColor rgb="FF1B1340"/>
+    <tabColor rgb="FF3D3D3D"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F21"/>

</xml_diff>